<commit_message>
feat: add playlist reordering and update content
- Implement manual reordering for playlist items
- Expand video library with new spiritual content
- Enrich curated playlists with additional videos
</commit_message>
<xml_diff>
--- a/Database.xlsx
+++ b/Database.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ashokgopalan/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7297A8B-7A0C-BF44-AEB1-A124FF2D5DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BDD052B9-4E87-D947-BAAE-380C4DE2A69A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="20440" xr2:uid="{26FF7FE2-E5E3-384C-ABF6-08C089761ADA}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="sample2" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sample2!$A$1:$D$956</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">sample2!$A$1:$D$1325</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4628" uniqueCount="3658">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5292" uniqueCount="4234">
   <si>
     <t>VideoID</t>
   </si>
@@ -11016,6 +11016,1734 @@
   </si>
   <si>
     <t>English|True Guru Guides From Experience|Inspirational Inspirational Clips||</t>
+  </si>
+  <si>
+    <t>EyBtOifZAys</t>
+  </si>
+  <si>
+    <t>Prayer at Dawn</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=EyBtOifZAys</t>
+  </si>
+  <si>
+    <t>hc2x64QAmvo</t>
+  </si>
+  <si>
+    <t>O God beautiful - Paramhansa Yogananda</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hc2x64QAmvo</t>
+  </si>
+  <si>
+    <t>IXY0CM83Jss</t>
+  </si>
+  <si>
+    <t>He Hari Sundara</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IXY0CM83Jss</t>
+  </si>
+  <si>
+    <t>Bju7gWiuZCU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Bju7gWiuZCU</t>
+  </si>
+  <si>
+    <t>hnTJwKDtHDA</t>
+  </si>
+  <si>
+    <t>God, Christ, Gurus</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hnTJwKDtHDA</t>
+  </si>
+  <si>
+    <t>wIKiFgsIWHs</t>
+  </si>
+  <si>
+    <t>Prayer at Noon</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=wIKiFgsIWHs</t>
+  </si>
+  <si>
+    <t>_rjI-ej-nGY</t>
+  </si>
+  <si>
+    <t>The Hound of Heaven</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_rjI-ej-nGY</t>
+  </si>
+  <si>
+    <t>FszBLKSeM28</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=FszBLKSeM28</t>
+  </si>
+  <si>
+    <t>DFH5PzhpFz8</t>
+  </si>
+  <si>
+    <t>Divine Mothers Song to the Devotee</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DFH5PzhpFz8</t>
+  </si>
+  <si>
+    <t>mhgwDjRjdFM</t>
+  </si>
+  <si>
+    <t>In the Temple of Silence</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mhgwDjRjdFM</t>
+  </si>
+  <si>
+    <t>L6h7v4TqZ4g</t>
+  </si>
+  <si>
+    <t>Song of India</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=L6h7v4TqZ4g</t>
+  </si>
+  <si>
+    <t>KFNdg7Q9YYs</t>
+  </si>
+  <si>
+    <t>Shanti Mundiray</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KFNdg7Q9YYs</t>
+  </si>
+  <si>
+    <t>3Z79qGEeQL8</t>
+  </si>
+  <si>
+    <t>Prayer at Eventide</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=3Z79qGEeQL8</t>
+  </si>
+  <si>
+    <t>j_8qDvlFmlU</t>
+  </si>
+  <si>
+    <t>I Will Be Thine Always</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=j_8qDvlFmlU</t>
+  </si>
+  <si>
+    <t>A0e9CPSym7k</t>
+  </si>
+  <si>
+    <t>Main Tera Hamesha</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=A0e9CPSym7k</t>
+  </si>
+  <si>
+    <t>iXP8mcipTgs</t>
+  </si>
+  <si>
+    <t>Do not dry the ocean of my Love - Paramhansa Yogananda</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=iXP8mcipTgs</t>
+  </si>
+  <si>
+    <t>upQUvPfT6W8</t>
+  </si>
+  <si>
+    <t>Prayer at Night</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=upQUvPfT6W8</t>
+  </si>
+  <si>
+    <t>MGa88qG0rt8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=MGa88qG0rt8</t>
+  </si>
+  <si>
+    <t>zV8x8uCoXc8</t>
+  </si>
+  <si>
+    <t>Who is in My Temple</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zV8x8uCoXc8</t>
+  </si>
+  <si>
+    <t>BgDz6DoeBg4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BgDz6DoeBg4</t>
+  </si>
+  <si>
+    <t>MHw4bfEjD2c</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=MHw4bfEjD2c</t>
+  </si>
+  <si>
+    <t>WMa7bIShNKI</t>
+  </si>
+  <si>
+    <t>In the Valley of Sorrow</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=WMa7bIShNKI</t>
+  </si>
+  <si>
+    <t>VlnAaiqtg8k</t>
+  </si>
+  <si>
+    <t>My Krishna is Blue</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VlnAaiqtg8k</t>
+  </si>
+  <si>
+    <t>OB6x3u7iipU</t>
+  </si>
+  <si>
+    <t>I Am the Sky</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=OB6x3u7iipU</t>
+  </si>
+  <si>
+    <t>lyuP_PgXCTM</t>
+  </si>
+  <si>
+    <t>Where is There Love</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=lyuP_PgXCTM</t>
+  </si>
+  <si>
+    <t>p1TSk004POw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=p1TSk004POw</t>
+  </si>
+  <si>
+    <t>4Q2sx4pCm0s</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=4Q2sx4pCm0s</t>
+  </si>
+  <si>
+    <t>IBWDk8g5C1g</t>
+  </si>
+  <si>
+    <t>Listen, Listen, Listen</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IBWDk8g5C1g</t>
+  </si>
+  <si>
+    <t>yBFJlXmngNA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yBFJlXmngNA</t>
+  </si>
+  <si>
+    <t>Ryc6TseZDkY</t>
+  </si>
+  <si>
+    <t>Today My Mind Has Dived</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Ryc6TseZDkY</t>
+  </si>
+  <si>
+    <t>BeXbDCqY3HY</t>
+  </si>
+  <si>
+    <t>Om Song</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BeXbDCqY3HY</t>
+  </si>
+  <si>
+    <t>IfwGaIW_Bmo</t>
+  </si>
+  <si>
+    <t>O Thou King of the Infinite</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=IfwGaIW_Bmo</t>
+  </si>
+  <si>
+    <t>Pn06BLdU67E</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Pn06BLdU67E</t>
+  </si>
+  <si>
+    <t>iNl48sdciKc</t>
+  </si>
+  <si>
+    <t>Divine Gypsy</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=iNl48sdciKc</t>
+  </si>
+  <si>
+    <t>KLJuiG8glFA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KLJuiG8glFA</t>
+  </si>
+  <si>
+    <t>WhGVZppb64M</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=WhGVZppb64M</t>
+  </si>
+  <si>
+    <t>vQbXGiVN7LU</t>
+  </si>
+  <si>
+    <t>O God Beautiful</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=vQbXGiVN7LU</t>
+  </si>
+  <si>
+    <t>ehZVfqD3WQs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ehZVfqD3WQs</t>
+  </si>
+  <si>
+    <t>oys07DpHR30</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=oys07DpHR30</t>
+  </si>
+  <si>
+    <t>kITE3vbsgT4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=kITE3vbsgT4</t>
+  </si>
+  <si>
+    <t>2GAQoi2OeDM</t>
+  </si>
+  <si>
+    <t>Door of My Heart</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2GAQoi2OeDM</t>
+  </si>
+  <si>
+    <t>aUa3A8Yvt8U</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aUa3A8Yvt8U</t>
+  </si>
+  <si>
+    <t>cu0mJ5fzLoY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=cu0mJ5fzLoY</t>
+  </si>
+  <si>
+    <t>9dr3gY_lf34</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9dr3gY_lf34</t>
+  </si>
+  <si>
+    <t>1R4_LzeiXK4</t>
+  </si>
+  <si>
+    <t>Light the Lamp of Thy Love</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=1R4_LzeiXK4</t>
+  </si>
+  <si>
+    <t>6yQKEHq4HAA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6yQKEHq4HAA</t>
+  </si>
+  <si>
+    <t>a0nOLb54y9s</t>
+  </si>
+  <si>
+    <t>Who Is in My Temple?</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=a0nOLb54y9s</t>
+  </si>
+  <si>
+    <t>NyAbtk4864c</t>
+  </si>
+  <si>
+    <t>Murali Krishna</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=NyAbtk4864c</t>
+  </si>
+  <si>
+    <t>yxF3_6JRsjo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yxF3_6JRsjo</t>
+  </si>
+  <si>
+    <t>PBMyZt_yURw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=PBMyZt_yURw</t>
+  </si>
+  <si>
+    <t>KqkQgkU2t6M</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KqkQgkU2t6M</t>
+  </si>
+  <si>
+    <t>q0BIshw_F10</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=q0BIshw_F10</t>
+  </si>
+  <si>
+    <t>62cSBt9bb4Q</t>
+  </si>
+  <si>
+    <t>Jaya Jaya Ma</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=62cSBt9bb4Q</t>
+  </si>
+  <si>
+    <t>H7Li5Yo2s9Q</t>
+  </si>
+  <si>
+    <t>Jai Guru</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=H7Li5Yo2s9Q</t>
+  </si>
+  <si>
+    <t>-AFByO1YL74</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=-AFByO1YL74</t>
+  </si>
+  <si>
+    <t>HDxFwX6kPbI</t>
+  </si>
+  <si>
+    <t>Radha Krishna Govinda</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=HDxFwX6kPbI</t>
+  </si>
+  <si>
+    <t>wbChJuu7CPM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=wbChJuu7CPM</t>
+  </si>
+  <si>
+    <t>fdqB5J32pX8</t>
+  </si>
+  <si>
+    <t>Guru Hamare</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=fdqB5J32pX8</t>
+  </si>
+  <si>
+    <t>VdugSeqC6Oo</t>
+  </si>
+  <si>
+    <t>Help Me Come Back</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VdugSeqC6Oo</t>
+  </si>
+  <si>
+    <t>SCCBfCeIvpI</t>
+  </si>
+  <si>
+    <t>Tero Naam</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=SCCBfCeIvpI</t>
+  </si>
+  <si>
+    <t>ZX2CbJvm2MQ</t>
+  </si>
+  <si>
+    <t>God, Krishna, Christ, Gurus</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ZX2CbJvm2MQ</t>
+  </si>
+  <si>
+    <t>urFqRZTIYmU</t>
+  </si>
+  <si>
+    <t>Om, Tat, Sat</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=urFqRZTIYmU</t>
+  </si>
+  <si>
+    <t>S312XGYA4t8</t>
+  </si>
+  <si>
+    <t>Namo, Namo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=S312XGYA4t8</t>
+  </si>
+  <si>
+    <t>aGT1iAkJMdA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aGT1iAkJMdA</t>
+  </si>
+  <si>
+    <t>LCpTZHPKBPw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=LCpTZHPKBPw</t>
+  </si>
+  <si>
+    <t>C65OWJ48RgU</t>
+  </si>
+  <si>
+    <t>Divine Mother’s Song to the Devotee</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=C65OWJ48RgU</t>
+  </si>
+  <si>
+    <t>d-j_6bDKlzI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=d-j_6bDKlzI</t>
+  </si>
+  <si>
+    <t>LbscWSheiNA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=LbscWSheiNA</t>
+  </si>
+  <si>
+    <t>2YF9W94JB3U</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2YF9W94JB3U</t>
+  </si>
+  <si>
+    <t>pncNctjTm1M</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=pncNctjTm1M</t>
+  </si>
+  <si>
+    <t>uT1dNRLmtu8</t>
+  </si>
+  <si>
+    <t>Polestar of My Life</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=uT1dNRLmtu8</t>
+  </si>
+  <si>
+    <t>JxO0Iml-fHk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=JxO0Iml-fHk</t>
+  </si>
+  <si>
+    <t>vfbI83oAZ8o</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=vfbI83oAZ8o</t>
+  </si>
+  <si>
+    <t>EHyxtdZvlY0</t>
+  </si>
+  <si>
+    <t>When Thy Song Flows Though Me</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=EHyxtdZvlY0</t>
+  </si>
+  <si>
+    <t>0AMd2PVkmAk</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=0AMd2PVkmAk</t>
+  </si>
+  <si>
+    <t>BPybvY2lDEw</t>
+  </si>
+  <si>
+    <t>Suno Mere Atma-Gan (At Thy Feet)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BPybvY2lDEw</t>
+  </si>
+  <si>
+    <t>9D1rd8hFj9s</t>
+  </si>
+  <si>
+    <t>Is Nind Se, Prabhu (From This Sleep, Lord)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9D1rd8hFj9s</t>
+  </si>
+  <si>
+    <t>_A94KMJDl7o</t>
+  </si>
+  <si>
+    <t>Dukh Ki Vadi Me (In the Valley of Sorrow)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_A94KMJDl7o</t>
+  </si>
+  <si>
+    <t>8RBBs6jeu_M</t>
+  </si>
+  <si>
+    <t>Nitya Navin Anand (Ever New Joy)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8RBBs6jeu_M</t>
+  </si>
+  <si>
+    <t>DfcNZfmdEDY</t>
+  </si>
+  <si>
+    <t>Shanti Mandir Me (In the Temple of Silence)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=DfcNZfmdEDY</t>
+  </si>
+  <si>
+    <t>G2wJnRwWoZc</t>
+  </si>
+  <si>
+    <t>Shyamal Krishna (Cloud-Colored Christ)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=G2wJnRwWoZc</t>
+  </si>
+  <si>
+    <t>ZUTbWsHy62o</t>
+  </si>
+  <si>
+    <t>Niras Na Karo Mere Prem Sagar Ko (Do Not Dry the Ocean of My Love)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ZUTbWsHy62o</t>
+  </si>
+  <si>
+    <t>fVOWVugDSxw</t>
+  </si>
+  <si>
+    <t>Ma, Tujhe Di Atma Ki Pukar (I Give You My Soul Call)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=fVOWVugDSxw</t>
+  </si>
+  <si>
+    <t>4bUcwYLB8kA</t>
+  </si>
+  <si>
+    <t>Kaun Hai Mere Mandir Me (Who is in My Temple)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=4bUcwYLB8kA</t>
+  </si>
+  <si>
+    <t>7nZM9mXjxfU</t>
+  </si>
+  <si>
+    <t>Nil Kamal Charan (Blue Lotus Feet)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7nZM9mXjxfU</t>
+  </si>
+  <si>
+    <t>N2aYWB1z2-k</t>
+  </si>
+  <si>
+    <t>Guru Stuti (Slokas) - He Bhagavan (Praise of the Guru - O Lord)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=N2aYWB1z2-k</t>
+  </si>
+  <si>
+    <t>2u1zIMyVxLw</t>
+  </si>
+  <si>
+    <t>Dhyan Karo (Meditate)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=2u1zIMyVxLw</t>
+  </si>
+  <si>
+    <t>BkCgGbqruiw</t>
+  </si>
+  <si>
+    <t>Bhaja Mana (Pray Night and Day)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BkCgGbqruiw</t>
+  </si>
+  <si>
+    <t>edlqMm-8OXk</t>
+  </si>
+  <si>
+    <t>Sri Guru Sharanam (I Surrender to the Guru)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=edlqMm-8OXk</t>
+  </si>
+  <si>
+    <t>krSz8ApD_KE</t>
+  </si>
+  <si>
+    <t>Krishna Stuti (Sloka) - Krishna Gopal Giridhari (Praise Lord Krishna - Victory to Krishna in...</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=krSz8ApD_KE</t>
+  </si>
+  <si>
+    <t>aBnUPM_sG2Y</t>
+  </si>
+  <si>
+    <t>Bhajan Karungi Tumhara (Lord, I Will Sing to Thee)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aBnUPM_sG2Y</t>
+  </si>
+  <si>
+    <t>XHgUOm4I5Po</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XHgUOm4I5Po</t>
+  </si>
+  <si>
+    <t>VDqKwucZLDY</t>
+  </si>
+  <si>
+    <t>Om Jai Jagadish Hare (Arati)</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=VDqKwucZLDY</t>
+  </si>
+  <si>
+    <t>jCEf3uDSreo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=jCEf3uDSreo</t>
+  </si>
+  <si>
+    <t>FmT8LxBhm7c</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=FmT8LxBhm7c</t>
+  </si>
+  <si>
+    <t>gENNZJit6Fc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gENNZJit6Fc</t>
+  </si>
+  <si>
+    <t>hH-J-Ms1_lA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hH-J-Ms1_lA</t>
+  </si>
+  <si>
+    <t>27SW7QNn0pg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=27SW7QNn0pg</t>
+  </si>
+  <si>
+    <t>XERunXHC-1Y</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XERunXHC-1Y</t>
+  </si>
+  <si>
+    <t>ucwxSN14GkY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ucwxSN14GkY</t>
+  </si>
+  <si>
+    <t>lLRwJlbokyM</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=lLRwJlbokyM</t>
+  </si>
+  <si>
+    <t>aYCXRprMhc8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=aYCXRprMhc8</t>
+  </si>
+  <si>
+    <t>e2PsAellOiI</t>
+  </si>
+  <si>
+    <t>They Have Heard Thy Name</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=e2PsAellOiI</t>
+  </si>
+  <si>
+    <t>yD6eVsvBf5Y</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=yD6eVsvBf5Y</t>
+  </si>
+  <si>
+    <t>k5wXErvuWZU</t>
+  </si>
+  <si>
+    <t>When My Dream's Dream is Done</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=k5wXErvuWZU</t>
+  </si>
+  <si>
+    <t>b1iXTbsaK60</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=b1iXTbsaK60</t>
+  </si>
+  <si>
+    <t>Au5yOzLvxnI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Au5yOzLvxnI</t>
+  </si>
+  <si>
+    <t>XO-VoGLqqSE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XO-VoGLqqSE</t>
+  </si>
+  <si>
+    <t>L2fNKupQTSQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=L2fNKupQTSQ</t>
+  </si>
+  <si>
+    <t>3-5XODAmWbA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=3-5XODAmWbA</t>
+  </si>
+  <si>
+    <t>sey0eWyRj94</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=sey0eWyRj94</t>
+  </si>
+  <si>
+    <t>KtV9EdJv9B0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KtV9EdJv9B0</t>
+  </si>
+  <si>
+    <t>Eiw1-Tgw6Uw</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Eiw1-Tgw6Uw</t>
+  </si>
+  <si>
+    <t>hZb8jkVwDcc</t>
+  </si>
+  <si>
+    <t>Will That Day Come to Me, Mother</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hZb8jkVwDcc</t>
+  </si>
+  <si>
+    <t>w4t5Rp7ksh0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=w4t5Rp7ksh0</t>
+  </si>
+  <si>
+    <t>9mZuIDNwLG8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=9mZuIDNwLG8</t>
+  </si>
+  <si>
+    <t>R3oN5u57Sdg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=R3oN5u57Sdg</t>
+  </si>
+  <si>
+    <t>nicK6v5xVkU</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=nicK6v5xVkU</t>
+  </si>
+  <si>
+    <t>3GJSJPBwAS8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=3GJSJPBwAS8</t>
+  </si>
+  <si>
+    <t>ESKVdyY4ZYY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=ESKVdyY4ZYY</t>
+  </si>
+  <si>
+    <t>_yx6ZK6EqOU</t>
+  </si>
+  <si>
+    <t>Ever-New Joy</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=_yx6ZK6EqOU</t>
+  </si>
+  <si>
+    <t>rRmCDUAG6Ek</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=rRmCDUAG6Ek</t>
+  </si>
+  <si>
+    <t>42frmqga5m0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=42frmqga5m0</t>
+  </si>
+  <si>
+    <t>KEvp3toAZeQ</t>
+  </si>
+  <si>
+    <t>Wake, Yet Wake, O My Saint</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=KEvp3toAZeQ</t>
+  </si>
+  <si>
+    <t>5XiAaGgGklQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5XiAaGgGklQ</t>
+  </si>
+  <si>
+    <t>Jdoz-xxcHKA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Jdoz-xxcHKA</t>
+  </si>
+  <si>
+    <t>7Y3W6bqoJ8k</t>
+  </si>
+  <si>
+    <t>He Who Knows</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=7Y3W6bqoJ8k</t>
+  </si>
+  <si>
+    <t>zgxviHCoyPs</t>
+  </si>
+  <si>
+    <t>Desire, My Great Enemy</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zgxviHCoyPs</t>
+  </si>
+  <si>
+    <t>a4ZxVychm90</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=a4ZxVychm90</t>
+  </si>
+  <si>
+    <t>Qn4Wmndg3vQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Qn4Wmndg3vQ</t>
+  </si>
+  <si>
+    <t>bYz_XyHsJKI</t>
+  </si>
+  <si>
+    <t>Polestar of My Life - O God Beautiful</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=bYz_XyHsJKI</t>
+  </si>
+  <si>
+    <t>jijHOc0R-4g</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=jijHOc0R-4g</t>
+  </si>
+  <si>
+    <t>jNqrEAWVLNE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=jNqrEAWVLNE</t>
+  </si>
+  <si>
+    <t>Nt3urPc2tkw</t>
+  </si>
+  <si>
+    <t>Satchidananda Guru</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Nt3urPc2tkw</t>
+  </si>
+  <si>
+    <t>zm2TRrZbLqI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=zm2TRrZbLqI</t>
+  </si>
+  <si>
+    <t>BdEtD_AN_Sc</t>
+  </si>
+  <si>
+    <t>Radhe Shyam</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=BdEtD_AN_Sc</t>
+  </si>
+  <si>
+    <t>XmQasAzmxCU</t>
+  </si>
+  <si>
+    <t>Blue Lotus Feet - Om Chant</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=XmQasAzmxCU</t>
+  </si>
+  <si>
+    <t>jI5iAnceXZ4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=jI5iAnceXZ4</t>
+  </si>
+  <si>
+    <t>6BDZL9e4zDg</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6BDZL9e4zDg</t>
+  </si>
+  <si>
+    <t>c5OBhhEf5FA</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=c5OBhhEf5FA</t>
+  </si>
+  <si>
+    <t>gx_VaV_mScU</t>
+  </si>
+  <si>
+    <t>Who Is in My Temple</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gx_VaV_mScU</t>
+  </si>
+  <si>
+    <t>COhHyD2U-r8</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=COhHyD2U-r8</t>
+  </si>
+  <si>
+    <t>z5xNm-VYLfM</t>
+  </si>
+  <si>
+    <t>Hare Krishna, Hare Ram</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=z5xNm-VYLfM</t>
+  </si>
+  <si>
+    <t>raQEPqlHzTQ</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=raQEPqlHzTQ</t>
+  </si>
+  <si>
+    <t>C--HVQLIxe0</t>
+  </si>
+  <si>
+    <t>He Bhagavan</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=C--HVQLIxe0</t>
+  </si>
+  <si>
+    <t>gj-dth2Crl0</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=gj-dth2Crl0</t>
+  </si>
+  <si>
+    <t>LbdlrkDveZM</t>
+  </si>
+  <si>
+    <t>Swami Ram Tirtha's Song</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=LbdlrkDveZM</t>
+  </si>
+  <si>
+    <t>UegOUQ97PWs</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UegOUQ97PWs</t>
+  </si>
+  <si>
+    <t>hrLrdTdTsr4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=hrLrdTdTsr4</t>
+  </si>
+  <si>
+    <t>c5C_4NTjiZs</t>
+  </si>
+  <si>
+    <t>Jai Guru - Radha Govinda Jai</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=c5C_4NTjiZs</t>
+  </si>
+  <si>
+    <t>kzncvlw781g</t>
+  </si>
+  <si>
+    <t>Aum Chant</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=kzncvlw781g</t>
+  </si>
+  <si>
+    <t>Fa0Q3XfS3Cc</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Fa0Q3XfS3Cc</t>
+  </si>
+  <si>
+    <t>5uK-ri-mMEE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=5uK-ri-mMEE</t>
+  </si>
+  <si>
+    <t>km2XWg7aHGs</t>
+  </si>
+  <si>
+    <t>Divine Mother's Song to the Devotee</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=km2XWg7aHGs</t>
+  </si>
+  <si>
+    <t>eqwc5nqtqbo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=eqwc5nqtqbo</t>
+  </si>
+  <si>
+    <t>MHjKi1oFeIY</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=MHjKi1oFeIY</t>
+  </si>
+  <si>
+    <t>AqFNf8QiRG4</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=AqFNf8QiRG4</t>
+  </si>
+  <si>
+    <t>8OXYnWbPSMo</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=8OXYnWbPSMo</t>
+  </si>
+  <si>
+    <t>UIq6YRA7HGE</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=UIq6YRA7HGE</t>
+  </si>
+  <si>
+    <t>SsIi9Ba4h2Y</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=SsIi9Ba4h2Y</t>
+  </si>
+  <si>
+    <t>P_QZSGjaK9Y</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=P_QZSGjaK9Y</t>
+  </si>
+  <si>
+    <t>mXZazhOSN84</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=mXZazhOSN84</t>
+  </si>
+  <si>
+    <t>Mj2w2WB9WwI</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=Mj2w2WB9WwI</t>
+  </si>
+  <si>
+    <t>s7redy0-Law</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=s7redy0-Law</t>
+  </si>
+  <si>
+    <t>6px3yz6gA-Y</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6px3yz6gA-Y</t>
+  </si>
+  <si>
+    <t>6bWOCm9OeTI</t>
+  </si>
+  <si>
+    <t>O God Beautiful - Aum Chant</t>
+  </si>
+  <si>
+    <t>https://www.youtube.com/watch?v=6bWOCm9OeTI</t>
+  </si>
+  <si>
+    <t>Prayer, Dawn|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Beautiful, Paramhansa, Yogananda|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Hari, Sundara|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>What, Lightning, Flash|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Christ, Gurus|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Prayer, Noon|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Hound, Heaven|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>CloudColored, Christ|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Mothers, Song, Devotee|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Temple, Silence|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Song, India|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Shanti, Mundiray|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Prayer, Eventide|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, Thine, Always|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Main, Tera, Hamesha|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Not, Dry, Ocean, Love, Paramhansa|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Prayer, Night|Mejda | Songs of My Heart|Kirtan</t>
+  </si>
+  <si>
+    <t>Deliver, From, Delusion|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Who, Temple|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thy, Feet|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Bubble, Make, Sea|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Valley, Sorrow|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Krishna, Blue|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Sky|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Where, There, Love|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>From, This, Sleep, Lord|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Land, Beyond, Dreams|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Listen|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Thy, Song, Flows, Through|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Today, Mind, Has, Dived|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Song|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, King, Infinite|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Kali|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Gypsy|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thousands, Suns|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Blue, Sky|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Beautiful|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Hymn, Brahma|I am the sky | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thy, Feet|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Bubble, Make, Sea|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Door, Heart|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>CloudColored, Christ|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Dawn, Chant|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Sri, Guru, Sharanam|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Light, Lamp, Thy, Love|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Sky|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Who, Temple|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Murali, Krishna|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Land, Beyond, Dreams|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Give, You, Soul, Call|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Thousands, Suns|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Art, Life|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Jaya|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Jai, Guru|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Blue, Sky|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Radha, Krishna, Govinda|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, Sing, Thy, Name|At Thy Feet | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Guru, Hamare|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>Help, Come, Back|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>Tero, Naam|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Krishna, Christ, Gurus|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>Tat, Sat|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>Namo|Guru Sharanam|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Art, Life|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Deliver, From, Delusion|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Mothers, Song, Devotee|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Krishna, Blue|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Where, There, Love|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>From, This, Sleep, Lord|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>CloudColored, Christ|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Polestar, Life|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Valley, Sorrow|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Blue, Lotus, Feet|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Thy, Song, Flows, Though|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Hymn, Brahma|Thou Art My Life | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Suno, Mere, AtmaGan, Thy, Feet|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Nind, Prabhu, From, This, Sleep|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Dukh, Vadi, Valley, Sorrow|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Nitya, Navin, Anand, Ever, New|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Shanti, Mandir, Temple, Silence|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Shyamal, Krishna, CloudColored, Christ|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Niras, Karo, Mere, Prem, Sagar|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Tujhe, Atma, Pukar, Give, You|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Kaun, Hai, Mere, Mandir, Who|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Nil, Kamal, Charan, Blue, Lotus|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Guru, Stuti, Slokas, Bhagavan, Praise|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Dhyan, Karo, Meditate|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Bhaja, Mana, Pray, Night, Day|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Sri, Guru, Sharanam, Surrender|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Krishna, Stuti, Sloka, Gopal, Giridhari|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Bhajan, Karungi, Tumhara, Lord, Will|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Hare, Krishna|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Jai, Jagadish, Hare, Arati|Shanti Mandir |Brahmacharini Mirabai|Kirtan</t>
+  </si>
+  <si>
+    <t>Land, Beyond, Dreams|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Blue, Lotus, Feet|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>From, This, Sleep, Lord|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Not, Dry, Ocean, Love|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Light, Lamp, Thy, Love|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Art, Life|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Valley, Sorrow|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Receive, Thy, Lap|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Deliver, From, Delusion|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>They, Have, Heard, Thy, Name|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Thy, Song, Flows, Through|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Dreams, Dream, Done|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Come, Listen, Soul, Song|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Give, You, Soul, Call|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, Thine, Always|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Where, There, Love|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Temple, Silence|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Wink, Has, Not, Touched, Eyes|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>I Am the Sky|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, King, Infinite|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, That, Day, Come, Mother|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Bubble, Make, Sea|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Hymn, Brahma|In the Land Beyond My Dreams | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>From, This, Sleep, Lord|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Land, Beyond, Dreams|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Come, Listen, Soul, Song|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Search, Him, Out, Secret|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>EverNew, Joy|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Dawn, Chant|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>What, Lightning, Flash|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Wake, Yet, Saint|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, That, Day, Come, Mother|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Blue, Sky|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Who, Knows|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Desire, Great, Enemy|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Dreams, Dream, Done|Where Golden Dreams Dwell | Instrumental|Kirtan</t>
+  </si>
+  <si>
+    <t>Hymn, Brahma|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Polestar, Life, God, Beautiful|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Spirit, Nature|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Dreams, Dream, Done|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Satchidananda, Guru|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Listen|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Radhe, Shyam|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Blue, Lotus, Feet, Chant|When My Dream's Dream is Done | SRF Nuns|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, Sing, Thy, Name|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Search, Him, Out, Secret|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Deliver, From, Delusion|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Who, Temple|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Spirit, Nature|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Hare, Krishna, Ram|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Valley, Sorrow|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Bhagavan|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Light, Lamp, Thy, Love|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Swami, Ram, Tirthas, Song|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Gypsy|I Will Sing Thy Name|Kirtan</t>
+  </si>
+  <si>
+    <t>Wink, Has, Not, Touched, Eyes|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Jai, Guru, Radha, Govinda|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Aum, Chant|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Gypsy|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Will, Thine, Always|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Divine, Mothers, Song, Devotee|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Thousands, Suns|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>They, Have, Heard, Thy, Name|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Sky|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Beautiful|The Divine Gypsy | Instrunmental|Kirtan</t>
+  </si>
+  <si>
+    <t>Jai, Guru|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>Thou, Art, Life|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>Door, Heart|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>When, Thy, Song, Flows, Through|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>Sky|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>Polestar, Life|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>Blue, Lotus, Feet|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
+  </si>
+  <si>
+    <t>God, Beautiful, Aum, Chant|When Thy Song Flows Through Me |SRF Monks|Kirtan</t>
   </si>
 </sst>
 </file>
@@ -11387,13 +13115,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE52D9B7-0D33-6C4B-ABD2-124A93043E14}">
-  <dimension ref="A1:D1159"/>
+  <dimension ref="A1:D1325"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="126" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34" customWidth="1"/>
     <col min="3" max="3" width="45.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -27619,8 +29348,2332 @@
         <v>3657</v>
       </c>
     </row>
+    <row r="1160" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1160" t="s">
+        <v>3658</v>
+      </c>
+      <c r="B1160" t="s">
+        <v>3659</v>
+      </c>
+      <c r="C1160" t="s">
+        <v>3660</v>
+      </c>
+      <c r="D1160" t="s">
+        <v>4068</v>
+      </c>
+    </row>
+    <row r="1161" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1161" t="s">
+        <v>3661</v>
+      </c>
+      <c r="B1161" t="s">
+        <v>3662</v>
+      </c>
+      <c r="C1161" t="s">
+        <v>3663</v>
+      </c>
+      <c r="D1161" t="s">
+        <v>4069</v>
+      </c>
+    </row>
+    <row r="1162" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1162" t="s">
+        <v>3664</v>
+      </c>
+      <c r="B1162" t="s">
+        <v>3665</v>
+      </c>
+      <c r="C1162" t="s">
+        <v>3666</v>
+      </c>
+      <c r="D1162" t="s">
+        <v>4070</v>
+      </c>
+    </row>
+    <row r="1163" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1163" t="s">
+        <v>3667</v>
+      </c>
+      <c r="B1163" t="s">
+        <v>3086</v>
+      </c>
+      <c r="C1163" t="s">
+        <v>3668</v>
+      </c>
+      <c r="D1163" t="s">
+        <v>4071</v>
+      </c>
+    </row>
+    <row r="1164" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1164" t="s">
+        <v>3669</v>
+      </c>
+      <c r="B1164" t="s">
+        <v>3670</v>
+      </c>
+      <c r="C1164" t="s">
+        <v>3671</v>
+      </c>
+      <c r="D1164" t="s">
+        <v>4072</v>
+      </c>
+    </row>
+    <row r="1165" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1165" t="s">
+        <v>3672</v>
+      </c>
+      <c r="B1165" t="s">
+        <v>3673</v>
+      </c>
+      <c r="C1165" t="s">
+        <v>3674</v>
+      </c>
+      <c r="D1165" t="s">
+        <v>4073</v>
+      </c>
+    </row>
+    <row r="1166" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1166" t="s">
+        <v>3675</v>
+      </c>
+      <c r="B1166" t="s">
+        <v>3676</v>
+      </c>
+      <c r="C1166" t="s">
+        <v>3677</v>
+      </c>
+      <c r="D1166" t="s">
+        <v>4074</v>
+      </c>
+    </row>
+    <row r="1167" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1167" t="s">
+        <v>3678</v>
+      </c>
+      <c r="B1167" t="s">
+        <v>3135</v>
+      </c>
+      <c r="C1167" t="s">
+        <v>3679</v>
+      </c>
+      <c r="D1167" t="s">
+        <v>4075</v>
+      </c>
+    </row>
+    <row r="1168" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1168" t="s">
+        <v>3680</v>
+      </c>
+      <c r="B1168" t="s">
+        <v>3681</v>
+      </c>
+      <c r="C1168" t="s">
+        <v>3682</v>
+      </c>
+      <c r="D1168" t="s">
+        <v>4076</v>
+      </c>
+    </row>
+    <row r="1169" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1169" t="s">
+        <v>3683</v>
+      </c>
+      <c r="B1169" t="s">
+        <v>3684</v>
+      </c>
+      <c r="C1169" t="s">
+        <v>3685</v>
+      </c>
+      <c r="D1169" t="s">
+        <v>4077</v>
+      </c>
+    </row>
+    <row r="1170" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1170" t="s">
+        <v>3686</v>
+      </c>
+      <c r="B1170" t="s">
+        <v>3687</v>
+      </c>
+      <c r="C1170" t="s">
+        <v>3688</v>
+      </c>
+      <c r="D1170" t="s">
+        <v>4078</v>
+      </c>
+    </row>
+    <row r="1171" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1171" t="s">
+        <v>3689</v>
+      </c>
+      <c r="B1171" t="s">
+        <v>3690</v>
+      </c>
+      <c r="C1171" t="s">
+        <v>3691</v>
+      </c>
+      <c r="D1171" t="s">
+        <v>4079</v>
+      </c>
+    </row>
+    <row r="1172" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1172" t="s">
+        <v>3692</v>
+      </c>
+      <c r="B1172" t="s">
+        <v>3693</v>
+      </c>
+      <c r="C1172" t="s">
+        <v>3694</v>
+      </c>
+      <c r="D1172" t="s">
+        <v>4080</v>
+      </c>
+    </row>
+    <row r="1173" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1173" t="s">
+        <v>3695</v>
+      </c>
+      <c r="B1173" t="s">
+        <v>3696</v>
+      </c>
+      <c r="C1173" t="s">
+        <v>3697</v>
+      </c>
+      <c r="D1173" t="s">
+        <v>4081</v>
+      </c>
+    </row>
+    <row r="1174" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1174" t="s">
+        <v>3698</v>
+      </c>
+      <c r="B1174" t="s">
+        <v>3699</v>
+      </c>
+      <c r="C1174" t="s">
+        <v>3700</v>
+      </c>
+      <c r="D1174" t="s">
+        <v>4082</v>
+      </c>
+    </row>
+    <row r="1175" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1175" t="s">
+        <v>3701</v>
+      </c>
+      <c r="B1175" t="s">
+        <v>3702</v>
+      </c>
+      <c r="C1175" t="s">
+        <v>3703</v>
+      </c>
+      <c r="D1175" t="s">
+        <v>4083</v>
+      </c>
+    </row>
+    <row r="1176" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1176" t="s">
+        <v>3704</v>
+      </c>
+      <c r="B1176" t="s">
+        <v>3705</v>
+      </c>
+      <c r="C1176" t="s">
+        <v>3706</v>
+      </c>
+      <c r="D1176" t="s">
+        <v>4084</v>
+      </c>
+    </row>
+    <row r="1177" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1177" t="s">
+        <v>3707</v>
+      </c>
+      <c r="B1177" t="s">
+        <v>3175</v>
+      </c>
+      <c r="C1177" t="s">
+        <v>3708</v>
+      </c>
+      <c r="D1177" t="s">
+        <v>4085</v>
+      </c>
+    </row>
+    <row r="1178" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1178" t="s">
+        <v>3709</v>
+      </c>
+      <c r="B1178" t="s">
+        <v>3710</v>
+      </c>
+      <c r="C1178" t="s">
+        <v>3711</v>
+      </c>
+      <c r="D1178" t="s">
+        <v>4086</v>
+      </c>
+    </row>
+    <row r="1179" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1179" t="s">
+        <v>3712</v>
+      </c>
+      <c r="B1179" t="s">
+        <v>3052</v>
+      </c>
+      <c r="C1179" t="s">
+        <v>3713</v>
+      </c>
+      <c r="D1179" t="s">
+        <v>4087</v>
+      </c>
+    </row>
+    <row r="1180" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1180" t="s">
+        <v>3714</v>
+      </c>
+      <c r="B1180" t="s">
+        <v>3038</v>
+      </c>
+      <c r="C1180" t="s">
+        <v>3715</v>
+      </c>
+      <c r="D1180" t="s">
+        <v>4088</v>
+      </c>
+    </row>
+    <row r="1181" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1181" t="s">
+        <v>3716</v>
+      </c>
+      <c r="B1181" t="s">
+        <v>3717</v>
+      </c>
+      <c r="C1181" t="s">
+        <v>3718</v>
+      </c>
+      <c r="D1181" t="s">
+        <v>4089</v>
+      </c>
+    </row>
+    <row r="1182" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1182" t="s">
+        <v>3719</v>
+      </c>
+      <c r="B1182" t="s">
+        <v>3720</v>
+      </c>
+      <c r="C1182" t="s">
+        <v>3721</v>
+      </c>
+      <c r="D1182" t="s">
+        <v>4090</v>
+      </c>
+    </row>
+    <row r="1183" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1183" t="s">
+        <v>3722</v>
+      </c>
+      <c r="B1183" t="s">
+        <v>3723</v>
+      </c>
+      <c r="C1183" t="s">
+        <v>3724</v>
+      </c>
+      <c r="D1183" t="s">
+        <v>4091</v>
+      </c>
+    </row>
+    <row r="1184" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1184" t="s">
+        <v>3725</v>
+      </c>
+      <c r="B1184" t="s">
+        <v>3726</v>
+      </c>
+      <c r="C1184" t="s">
+        <v>3727</v>
+      </c>
+      <c r="D1184" t="s">
+        <v>4092</v>
+      </c>
+    </row>
+    <row r="1185" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1185" t="s">
+        <v>3728</v>
+      </c>
+      <c r="B1185" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C1185" t="s">
+        <v>3729</v>
+      </c>
+      <c r="D1185" t="s">
+        <v>4093</v>
+      </c>
+    </row>
+    <row r="1186" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1186" t="s">
+        <v>3730</v>
+      </c>
+      <c r="B1186" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1186" t="s">
+        <v>3731</v>
+      </c>
+      <c r="D1186" t="s">
+        <v>4094</v>
+      </c>
+    </row>
+    <row r="1187" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1187" t="s">
+        <v>3732</v>
+      </c>
+      <c r="B1187" t="s">
+        <v>3733</v>
+      </c>
+      <c r="C1187" t="s">
+        <v>3734</v>
+      </c>
+      <c r="D1187" t="s">
+        <v>4095</v>
+      </c>
+    </row>
+    <row r="1188" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1188" t="s">
+        <v>3735</v>
+      </c>
+      <c r="B1188" t="s">
+        <v>3047</v>
+      </c>
+      <c r="C1188" t="s">
+        <v>3736</v>
+      </c>
+      <c r="D1188" t="s">
+        <v>4096</v>
+      </c>
+    </row>
+    <row r="1189" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1189" t="s">
+        <v>3737</v>
+      </c>
+      <c r="B1189" t="s">
+        <v>3738</v>
+      </c>
+      <c r="C1189" t="s">
+        <v>3739</v>
+      </c>
+      <c r="D1189" t="s">
+        <v>4097</v>
+      </c>
+    </row>
+    <row r="1190" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1190" t="s">
+        <v>3740</v>
+      </c>
+      <c r="B1190" t="s">
+        <v>3741</v>
+      </c>
+      <c r="C1190" t="s">
+        <v>3742</v>
+      </c>
+      <c r="D1190" t="s">
+        <v>4098</v>
+      </c>
+    </row>
+    <row r="1191" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1191" t="s">
+        <v>3743</v>
+      </c>
+      <c r="B1191" t="s">
+        <v>3744</v>
+      </c>
+      <c r="C1191" t="s">
+        <v>3745</v>
+      </c>
+      <c r="D1191" t="s">
+        <v>4099</v>
+      </c>
+    </row>
+    <row r="1192" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1192" t="s">
+        <v>3746</v>
+      </c>
+      <c r="B1192" t="s">
+        <v>3023</v>
+      </c>
+      <c r="C1192" t="s">
+        <v>3747</v>
+      </c>
+      <c r="D1192" t="s">
+        <v>4100</v>
+      </c>
+    </row>
+    <row r="1193" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1193" t="s">
+        <v>3748</v>
+      </c>
+      <c r="B1193" t="s">
+        <v>3749</v>
+      </c>
+      <c r="C1193" t="s">
+        <v>3750</v>
+      </c>
+      <c r="D1193" t="s">
+        <v>4101</v>
+      </c>
+    </row>
+    <row r="1194" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1194" t="s">
+        <v>3751</v>
+      </c>
+      <c r="B1194" t="s">
+        <v>3132</v>
+      </c>
+      <c r="C1194" t="s">
+        <v>3752</v>
+      </c>
+      <c r="D1194" t="s">
+        <v>4102</v>
+      </c>
+    </row>
+    <row r="1195" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1195" t="s">
+        <v>3753</v>
+      </c>
+      <c r="B1195" t="s">
+        <v>3124</v>
+      </c>
+      <c r="C1195" t="s">
+        <v>3754</v>
+      </c>
+      <c r="D1195" t="s">
+        <v>4103</v>
+      </c>
+    </row>
+    <row r="1196" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1196" t="s">
+        <v>3755</v>
+      </c>
+      <c r="B1196" t="s">
+        <v>3756</v>
+      </c>
+      <c r="C1196" t="s">
+        <v>3757</v>
+      </c>
+      <c r="D1196" t="s">
+        <v>4104</v>
+      </c>
+    </row>
+    <row r="1197" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1197" t="s">
+        <v>3758</v>
+      </c>
+      <c r="B1197" t="s">
+        <v>3014</v>
+      </c>
+      <c r="C1197" t="s">
+        <v>3759</v>
+      </c>
+      <c r="D1197" t="s">
+        <v>4105</v>
+      </c>
+    </row>
+    <row r="1198" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1198" t="s">
+        <v>3760</v>
+      </c>
+      <c r="B1198" t="s">
+        <v>3052</v>
+      </c>
+      <c r="C1198" t="s">
+        <v>3761</v>
+      </c>
+      <c r="D1198" t="s">
+        <v>4106</v>
+      </c>
+    </row>
+    <row r="1199" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1199" t="s">
+        <v>3762</v>
+      </c>
+      <c r="B1199" t="s">
+        <v>3038</v>
+      </c>
+      <c r="C1199" t="s">
+        <v>3763</v>
+      </c>
+      <c r="D1199" t="s">
+        <v>4107</v>
+      </c>
+    </row>
+    <row r="1200" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1200" t="s">
+        <v>3764</v>
+      </c>
+      <c r="B1200" t="s">
+        <v>3765</v>
+      </c>
+      <c r="C1200" t="s">
+        <v>3766</v>
+      </c>
+      <c r="D1200" t="s">
+        <v>4108</v>
+      </c>
+    </row>
+    <row r="1201" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1201" t="s">
+        <v>3767</v>
+      </c>
+      <c r="B1201" t="s">
+        <v>3135</v>
+      </c>
+      <c r="C1201" t="s">
+        <v>3768</v>
+      </c>
+      <c r="D1201" t="s">
+        <v>4109</v>
+      </c>
+    </row>
+    <row r="1202" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1202" t="s">
+        <v>3769</v>
+      </c>
+      <c r="B1202" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C1202" t="s">
+        <v>3770</v>
+      </c>
+      <c r="D1202" t="s">
+        <v>4110</v>
+      </c>
+    </row>
+    <row r="1203" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1203" t="s">
+        <v>3771</v>
+      </c>
+      <c r="B1203" t="s">
+        <v>3055</v>
+      </c>
+      <c r="C1203" t="s">
+        <v>3772</v>
+      </c>
+      <c r="D1203" t="s">
+        <v>4111</v>
+      </c>
+    </row>
+    <row r="1204" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1204" t="s">
+        <v>3773</v>
+      </c>
+      <c r="B1204" t="s">
+        <v>3774</v>
+      </c>
+      <c r="C1204" t="s">
+        <v>3775</v>
+      </c>
+      <c r="D1204" t="s">
+        <v>4112</v>
+      </c>
+    </row>
+    <row r="1205" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1205" t="s">
+        <v>3776</v>
+      </c>
+      <c r="B1205" t="s">
+        <v>3723</v>
+      </c>
+      <c r="C1205" t="s">
+        <v>3777</v>
+      </c>
+      <c r="D1205" t="s">
+        <v>4113</v>
+      </c>
+    </row>
+    <row r="1206" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1206" t="s">
+        <v>3778</v>
+      </c>
+      <c r="B1206" t="s">
+        <v>3779</v>
+      </c>
+      <c r="C1206" t="s">
+        <v>3780</v>
+      </c>
+      <c r="D1206" t="s">
+        <v>4114</v>
+      </c>
+    </row>
+    <row r="1207" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1207" t="s">
+        <v>3781</v>
+      </c>
+      <c r="B1207" t="s">
+        <v>3782</v>
+      </c>
+      <c r="C1207" t="s">
+        <v>3783</v>
+      </c>
+      <c r="D1207" t="s">
+        <v>4115</v>
+      </c>
+    </row>
+    <row r="1208" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1208" t="s">
+        <v>3784</v>
+      </c>
+      <c r="B1208" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1208" t="s">
+        <v>3785</v>
+      </c>
+      <c r="D1208" t="s">
+        <v>4116</v>
+      </c>
+    </row>
+    <row r="1209" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1209" t="s">
+        <v>3786</v>
+      </c>
+      <c r="B1209" t="s">
+        <v>3080</v>
+      </c>
+      <c r="C1209" t="s">
+        <v>3787</v>
+      </c>
+      <c r="D1209" t="s">
+        <v>4117</v>
+      </c>
+    </row>
+    <row r="1210" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1210" t="s">
+        <v>3788</v>
+      </c>
+      <c r="B1210" t="s">
+        <v>3132</v>
+      </c>
+      <c r="C1210" t="s">
+        <v>3789</v>
+      </c>
+      <c r="D1210" t="s">
+        <v>4118</v>
+      </c>
+    </row>
+    <row r="1211" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1211" t="s">
+        <v>3790</v>
+      </c>
+      <c r="B1211" t="s">
+        <v>3035</v>
+      </c>
+      <c r="C1211" t="s">
+        <v>3791</v>
+      </c>
+      <c r="D1211" t="s">
+        <v>4119</v>
+      </c>
+    </row>
+    <row r="1212" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1212" t="s">
+        <v>3792</v>
+      </c>
+      <c r="B1212" t="s">
+        <v>3793</v>
+      </c>
+      <c r="C1212" t="s">
+        <v>3794</v>
+      </c>
+      <c r="D1212" t="s">
+        <v>4120</v>
+      </c>
+    </row>
+    <row r="1213" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1213" t="s">
+        <v>3795</v>
+      </c>
+      <c r="B1213" t="s">
+        <v>3796</v>
+      </c>
+      <c r="C1213" t="s">
+        <v>3797</v>
+      </c>
+      <c r="D1213" t="s">
+        <v>4121</v>
+      </c>
+    </row>
+    <row r="1214" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1214" t="s">
+        <v>3798</v>
+      </c>
+      <c r="B1214" t="s">
+        <v>3124</v>
+      </c>
+      <c r="C1214" t="s">
+        <v>3799</v>
+      </c>
+      <c r="D1214" t="s">
+        <v>4122</v>
+      </c>
+    </row>
+    <row r="1215" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1215" t="s">
+        <v>3800</v>
+      </c>
+      <c r="B1215" t="s">
+        <v>3801</v>
+      </c>
+      <c r="C1215" t="s">
+        <v>3802</v>
+      </c>
+      <c r="D1215" t="s">
+        <v>4123</v>
+      </c>
+    </row>
+    <row r="1216" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1216" t="s">
+        <v>3803</v>
+      </c>
+      <c r="B1216" t="s">
+        <v>3169</v>
+      </c>
+      <c r="C1216" t="s">
+        <v>3804</v>
+      </c>
+      <c r="D1216" t="s">
+        <v>4124</v>
+      </c>
+    </row>
+    <row r="1217" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1217" t="s">
+        <v>3805</v>
+      </c>
+      <c r="B1217" t="s">
+        <v>3806</v>
+      </c>
+      <c r="C1217" t="s">
+        <v>3807</v>
+      </c>
+      <c r="D1217" t="s">
+        <v>4125</v>
+      </c>
+    </row>
+    <row r="1218" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1218" t="s">
+        <v>3808</v>
+      </c>
+      <c r="B1218" t="s">
+        <v>3809</v>
+      </c>
+      <c r="C1218" t="s">
+        <v>3810</v>
+      </c>
+      <c r="D1218" t="s">
+        <v>4126</v>
+      </c>
+    </row>
+    <row r="1219" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1219" t="s">
+        <v>3811</v>
+      </c>
+      <c r="B1219" t="s">
+        <v>3812</v>
+      </c>
+      <c r="C1219" t="s">
+        <v>3813</v>
+      </c>
+      <c r="D1219" t="s">
+        <v>4127</v>
+      </c>
+    </row>
+    <row r="1220" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1220" t="s">
+        <v>3814</v>
+      </c>
+      <c r="B1220" t="s">
+        <v>3815</v>
+      </c>
+      <c r="C1220" t="s">
+        <v>3816</v>
+      </c>
+      <c r="D1220" t="s">
+        <v>4128</v>
+      </c>
+    </row>
+    <row r="1221" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1221" t="s">
+        <v>3817</v>
+      </c>
+      <c r="B1221" t="s">
+        <v>3818</v>
+      </c>
+      <c r="C1221" t="s">
+        <v>3819</v>
+      </c>
+      <c r="D1221" t="s">
+        <v>4129</v>
+      </c>
+    </row>
+    <row r="1222" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1222" t="s">
+        <v>3820</v>
+      </c>
+      <c r="B1222" t="s">
+        <v>3821</v>
+      </c>
+      <c r="C1222" t="s">
+        <v>3822</v>
+      </c>
+      <c r="D1222" t="s">
+        <v>4130</v>
+      </c>
+    </row>
+    <row r="1223" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1223" t="s">
+        <v>3823</v>
+      </c>
+      <c r="B1223" t="s">
+        <v>3035</v>
+      </c>
+      <c r="C1223" t="s">
+        <v>3824</v>
+      </c>
+      <c r="D1223" t="s">
+        <v>4131</v>
+      </c>
+    </row>
+    <row r="1224" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1224" t="s">
+        <v>3825</v>
+      </c>
+      <c r="B1224" t="s">
+        <v>3175</v>
+      </c>
+      <c r="C1224" t="s">
+        <v>3826</v>
+      </c>
+      <c r="D1224" t="s">
+        <v>4132</v>
+      </c>
+    </row>
+    <row r="1225" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1225" t="s">
+        <v>3827</v>
+      </c>
+      <c r="B1225" t="s">
+        <v>3828</v>
+      </c>
+      <c r="C1225" t="s">
+        <v>3829</v>
+      </c>
+      <c r="D1225" t="s">
+        <v>4133</v>
+      </c>
+    </row>
+    <row r="1226" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1226" t="s">
+        <v>3830</v>
+      </c>
+      <c r="B1226" t="s">
+        <v>3032</v>
+      </c>
+      <c r="C1226" t="s">
+        <v>3831</v>
+      </c>
+      <c r="D1226" t="s">
+        <v>4134</v>
+      </c>
+    </row>
+    <row r="1227" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1227" t="s">
+        <v>3832</v>
+      </c>
+      <c r="B1227" t="s">
+        <v>3147</v>
+      </c>
+      <c r="C1227" t="s">
+        <v>3833</v>
+      </c>
+      <c r="D1227" t="s">
+        <v>4135</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1228" t="s">
+        <v>3834</v>
+      </c>
+      <c r="B1228" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C1228" t="s">
+        <v>3835</v>
+      </c>
+      <c r="D1228" t="s">
+        <v>4136</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1229" t="s">
+        <v>3836</v>
+      </c>
+      <c r="B1229" t="s">
+        <v>3135</v>
+      </c>
+      <c r="C1229" t="s">
+        <v>3837</v>
+      </c>
+      <c r="D1229" t="s">
+        <v>4137</v>
+      </c>
+    </row>
+    <row r="1230" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1230" t="s">
+        <v>3838</v>
+      </c>
+      <c r="B1230" t="s">
+        <v>3839</v>
+      </c>
+      <c r="C1230" t="s">
+        <v>3840</v>
+      </c>
+      <c r="D1230" t="s">
+        <v>4138</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1231" t="s">
+        <v>3841</v>
+      </c>
+      <c r="B1231" t="s">
+        <v>3717</v>
+      </c>
+      <c r="C1231" t="s">
+        <v>3842</v>
+      </c>
+      <c r="D1231" t="s">
+        <v>4139</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1232" t="s">
+        <v>3843</v>
+      </c>
+      <c r="B1232" t="s">
+        <v>3061</v>
+      </c>
+      <c r="C1232" t="s">
+        <v>3844</v>
+      </c>
+      <c r="D1232" t="s">
+        <v>4140</v>
+      </c>
+    </row>
+    <row r="1233" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1233" t="s">
+        <v>3845</v>
+      </c>
+      <c r="B1233" t="s">
+        <v>3846</v>
+      </c>
+      <c r="C1233" t="s">
+        <v>3847</v>
+      </c>
+      <c r="D1233" t="s">
+        <v>4141</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1234" t="s">
+        <v>3848</v>
+      </c>
+      <c r="B1234" t="s">
+        <v>3014</v>
+      </c>
+      <c r="C1234" t="s">
+        <v>3849</v>
+      </c>
+      <c r="D1234" t="s">
+        <v>4142</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1235" t="s">
+        <v>3850</v>
+      </c>
+      <c r="B1235" t="s">
+        <v>3851</v>
+      </c>
+      <c r="C1235" t="s">
+        <v>3852</v>
+      </c>
+      <c r="D1235" t="s">
+        <v>4143</v>
+      </c>
+    </row>
+    <row r="1236" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1236" t="s">
+        <v>3853</v>
+      </c>
+      <c r="B1236" t="s">
+        <v>3854</v>
+      </c>
+      <c r="C1236" t="s">
+        <v>3855</v>
+      </c>
+      <c r="D1236" t="s">
+        <v>4144</v>
+      </c>
+    </row>
+    <row r="1237" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1237" t="s">
+        <v>3856</v>
+      </c>
+      <c r="B1237" t="s">
+        <v>3857</v>
+      </c>
+      <c r="C1237" t="s">
+        <v>3858</v>
+      </c>
+      <c r="D1237" t="s">
+        <v>4145</v>
+      </c>
+    </row>
+    <row r="1238" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1238" t="s">
+        <v>3859</v>
+      </c>
+      <c r="B1238" t="s">
+        <v>3860</v>
+      </c>
+      <c r="C1238" t="s">
+        <v>3861</v>
+      </c>
+      <c r="D1238" t="s">
+        <v>4146</v>
+      </c>
+    </row>
+    <row r="1239" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1239" t="s">
+        <v>3862</v>
+      </c>
+      <c r="B1239" t="s">
+        <v>3863</v>
+      </c>
+      <c r="C1239" t="s">
+        <v>3864</v>
+      </c>
+      <c r="D1239" t="s">
+        <v>4147</v>
+      </c>
+    </row>
+    <row r="1240" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1240" t="s">
+        <v>3865</v>
+      </c>
+      <c r="B1240" t="s">
+        <v>3866</v>
+      </c>
+      <c r="C1240" t="s">
+        <v>3867</v>
+      </c>
+      <c r="D1240" t="s">
+        <v>4148</v>
+      </c>
+    </row>
+    <row r="1241" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1241" t="s">
+        <v>3868</v>
+      </c>
+      <c r="B1241" t="s">
+        <v>3869</v>
+      </c>
+      <c r="C1241" t="s">
+        <v>3870</v>
+      </c>
+      <c r="D1241" t="s">
+        <v>4149</v>
+      </c>
+    </row>
+    <row r="1242" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1242" t="s">
+        <v>3871</v>
+      </c>
+      <c r="B1242" t="s">
+        <v>3872</v>
+      </c>
+      <c r="C1242" t="s">
+        <v>3873</v>
+      </c>
+      <c r="D1242" t="s">
+        <v>4150</v>
+      </c>
+    </row>
+    <row r="1243" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1243" t="s">
+        <v>3874</v>
+      </c>
+      <c r="B1243" t="s">
+        <v>3875</v>
+      </c>
+      <c r="C1243" t="s">
+        <v>3876</v>
+      </c>
+      <c r="D1243" t="s">
+        <v>4151</v>
+      </c>
+    </row>
+    <row r="1244" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1244" t="s">
+        <v>3877</v>
+      </c>
+      <c r="B1244" t="s">
+        <v>3878</v>
+      </c>
+      <c r="C1244" t="s">
+        <v>3879</v>
+      </c>
+      <c r="D1244" t="s">
+        <v>4152</v>
+      </c>
+    </row>
+    <row r="1245" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1245" t="s">
+        <v>3880</v>
+      </c>
+      <c r="B1245" t="s">
+        <v>3881</v>
+      </c>
+      <c r="C1245" t="s">
+        <v>3882</v>
+      </c>
+      <c r="D1245" t="s">
+        <v>4153</v>
+      </c>
+    </row>
+    <row r="1246" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1246" t="s">
+        <v>3883</v>
+      </c>
+      <c r="B1246" t="s">
+        <v>3884</v>
+      </c>
+      <c r="C1246" t="s">
+        <v>3885</v>
+      </c>
+      <c r="D1246" t="s">
+        <v>4154</v>
+      </c>
+    </row>
+    <row r="1247" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1247" t="s">
+        <v>3886</v>
+      </c>
+      <c r="B1247" t="s">
+        <v>3887</v>
+      </c>
+      <c r="C1247" t="s">
+        <v>3888</v>
+      </c>
+      <c r="D1247" t="s">
+        <v>4155</v>
+      </c>
+    </row>
+    <row r="1248" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1248" t="s">
+        <v>3889</v>
+      </c>
+      <c r="B1248" t="s">
+        <v>3890</v>
+      </c>
+      <c r="C1248" t="s">
+        <v>3891</v>
+      </c>
+      <c r="D1248" t="s">
+        <v>4156</v>
+      </c>
+    </row>
+    <row r="1249" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1249" t="s">
+        <v>3892</v>
+      </c>
+      <c r="B1249" t="s">
+        <v>3893</v>
+      </c>
+      <c r="C1249" t="s">
+        <v>3894</v>
+      </c>
+      <c r="D1249" t="s">
+        <v>4157</v>
+      </c>
+    </row>
+    <row r="1250" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1250" t="s">
+        <v>3895</v>
+      </c>
+      <c r="B1250" t="s">
+        <v>3896</v>
+      </c>
+      <c r="C1250" t="s">
+        <v>3897</v>
+      </c>
+      <c r="D1250" t="s">
+        <v>4158</v>
+      </c>
+    </row>
+    <row r="1251" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1251" t="s">
+        <v>3898</v>
+      </c>
+      <c r="B1251" t="s">
+        <v>3144</v>
+      </c>
+      <c r="C1251" t="s">
+        <v>3899</v>
+      </c>
+      <c r="D1251" t="s">
+        <v>4159</v>
+      </c>
+    </row>
+    <row r="1252" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1252" t="s">
+        <v>3900</v>
+      </c>
+      <c r="B1252" t="s">
+        <v>3901</v>
+      </c>
+      <c r="C1252" t="s">
+        <v>3902</v>
+      </c>
+      <c r="D1252" t="s">
+        <v>4160</v>
+      </c>
+    </row>
+    <row r="1253" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1253" t="s">
+        <v>3903</v>
+      </c>
+      <c r="B1253" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1253" t="s">
+        <v>3904</v>
+      </c>
+      <c r="D1253" t="s">
+        <v>4161</v>
+      </c>
+    </row>
+    <row r="1254" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1254" t="s">
+        <v>3905</v>
+      </c>
+      <c r="B1254" t="s">
+        <v>3061</v>
+      </c>
+      <c r="C1254" t="s">
+        <v>3906</v>
+      </c>
+      <c r="D1254" t="s">
+        <v>4162</v>
+      </c>
+    </row>
+    <row r="1255" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1255" t="s">
+        <v>3907</v>
+      </c>
+      <c r="B1255" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C1255" t="s">
+        <v>3908</v>
+      </c>
+      <c r="D1255" t="s">
+        <v>4163</v>
+      </c>
+    </row>
+    <row r="1256" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1256" t="s">
+        <v>3909</v>
+      </c>
+      <c r="B1256" t="s">
+        <v>3026</v>
+      </c>
+      <c r="C1256" t="s">
+        <v>3910</v>
+      </c>
+      <c r="D1256" t="s">
+        <v>4164</v>
+      </c>
+    </row>
+    <row r="1257" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1257" t="s">
+        <v>3911</v>
+      </c>
+      <c r="B1257" t="s">
+        <v>3774</v>
+      </c>
+      <c r="C1257" t="s">
+        <v>3912</v>
+      </c>
+      <c r="D1257" t="s">
+        <v>4165</v>
+      </c>
+    </row>
+    <row r="1258" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1258" t="s">
+        <v>3913</v>
+      </c>
+      <c r="B1258" t="s">
+        <v>3035</v>
+      </c>
+      <c r="C1258" t="s">
+        <v>3914</v>
+      </c>
+      <c r="D1258" t="s">
+        <v>4166</v>
+      </c>
+    </row>
+    <row r="1259" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1259" t="s">
+        <v>3915</v>
+      </c>
+      <c r="B1259" t="s">
+        <v>3717</v>
+      </c>
+      <c r="C1259" t="s">
+        <v>3916</v>
+      </c>
+      <c r="D1259" t="s">
+        <v>4167</v>
+      </c>
+    </row>
+    <row r="1260" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1260" t="s">
+        <v>3917</v>
+      </c>
+      <c r="B1260" t="s">
+        <v>3138</v>
+      </c>
+      <c r="C1260" t="s">
+        <v>3918</v>
+      </c>
+      <c r="D1260" t="s">
+        <v>4168</v>
+      </c>
+    </row>
+    <row r="1261" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1261" t="s">
+        <v>3919</v>
+      </c>
+      <c r="B1261" t="s">
+        <v>3175</v>
+      </c>
+      <c r="C1261" t="s">
+        <v>3920</v>
+      </c>
+      <c r="D1261" t="s">
+        <v>4169</v>
+      </c>
+    </row>
+    <row r="1262" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1262" t="s">
+        <v>3921</v>
+      </c>
+      <c r="B1262" t="s">
+        <v>3922</v>
+      </c>
+      <c r="C1262" t="s">
+        <v>3923</v>
+      </c>
+      <c r="D1262" t="s">
+        <v>4170</v>
+      </c>
+    </row>
+    <row r="1263" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1263" t="s">
+        <v>3924</v>
+      </c>
+      <c r="B1263" t="s">
+        <v>3047</v>
+      </c>
+      <c r="C1263" t="s">
+        <v>3925</v>
+      </c>
+      <c r="D1263" t="s">
+        <v>4171</v>
+      </c>
+    </row>
+    <row r="1264" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1264" t="s">
+        <v>3926</v>
+      </c>
+      <c r="B1264" t="s">
+        <v>3927</v>
+      </c>
+      <c r="C1264" t="s">
+        <v>3928</v>
+      </c>
+      <c r="D1264" t="s">
+        <v>4172</v>
+      </c>
+    </row>
+    <row r="1265" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1265" t="s">
+        <v>3929</v>
+      </c>
+      <c r="B1265" t="s">
+        <v>3117</v>
+      </c>
+      <c r="C1265" t="s">
+        <v>3930</v>
+      </c>
+      <c r="D1265" t="s">
+        <v>4173</v>
+      </c>
+    </row>
+    <row r="1266" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1266" t="s">
+        <v>3931</v>
+      </c>
+      <c r="B1266" t="s">
+        <v>3080</v>
+      </c>
+      <c r="C1266" t="s">
+        <v>3932</v>
+      </c>
+      <c r="D1266" t="s">
+        <v>4174</v>
+      </c>
+    </row>
+    <row r="1267" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1267" t="s">
+        <v>3933</v>
+      </c>
+      <c r="B1267" t="s">
+        <v>3696</v>
+      </c>
+      <c r="C1267" t="s">
+        <v>3934</v>
+      </c>
+      <c r="D1267" t="s">
+        <v>4175</v>
+      </c>
+    </row>
+    <row r="1268" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1268" t="s">
+        <v>3935</v>
+      </c>
+      <c r="B1268" t="s">
+        <v>3726</v>
+      </c>
+      <c r="C1268" t="s">
+        <v>3936</v>
+      </c>
+      <c r="D1268" t="s">
+        <v>4176</v>
+      </c>
+    </row>
+    <row r="1269" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1269" t="s">
+        <v>3937</v>
+      </c>
+      <c r="B1269" t="s">
+        <v>3684</v>
+      </c>
+      <c r="C1269" t="s">
+        <v>3938</v>
+      </c>
+      <c r="D1269" t="s">
+        <v>4177</v>
+      </c>
+    </row>
+    <row r="1270" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1270" t="s">
+        <v>3939</v>
+      </c>
+      <c r="B1270" t="s">
+        <v>3089</v>
+      </c>
+      <c r="C1270" t="s">
+        <v>3940</v>
+      </c>
+      <c r="D1270" t="s">
+        <v>4178</v>
+      </c>
+    </row>
+    <row r="1271" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1271" t="s">
+        <v>3941</v>
+      </c>
+      <c r="B1271" t="s">
+        <v>3723</v>
+      </c>
+      <c r="C1271" t="s">
+        <v>3942</v>
+      </c>
+      <c r="D1271" t="s">
+        <v>4179</v>
+      </c>
+    </row>
+    <row r="1272" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1272" t="s">
+        <v>3943</v>
+      </c>
+      <c r="B1272" t="s">
+        <v>3744</v>
+      </c>
+      <c r="C1272" t="s">
+        <v>3944</v>
+      </c>
+      <c r="D1272" t="s">
+        <v>4180</v>
+      </c>
+    </row>
+    <row r="1273" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1273" t="s">
+        <v>3945</v>
+      </c>
+      <c r="B1273" t="s">
+        <v>3946</v>
+      </c>
+      <c r="C1273" t="s">
+        <v>3947</v>
+      </c>
+      <c r="D1273" t="s">
+        <v>4181</v>
+      </c>
+    </row>
+    <row r="1274" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1274" t="s">
+        <v>3948</v>
+      </c>
+      <c r="B1274" t="s">
+        <v>3038</v>
+      </c>
+      <c r="C1274" t="s">
+        <v>3949</v>
+      </c>
+      <c r="D1274" t="s">
+        <v>4182</v>
+      </c>
+    </row>
+    <row r="1275" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1275" t="s">
+        <v>3950</v>
+      </c>
+      <c r="B1275" t="s">
+        <v>3014</v>
+      </c>
+      <c r="C1275" t="s">
+        <v>3951</v>
+      </c>
+      <c r="D1275" t="s">
+        <v>4183</v>
+      </c>
+    </row>
+    <row r="1276" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1276" t="s">
+        <v>3952</v>
+      </c>
+      <c r="B1276" t="s">
+        <v>3141</v>
+      </c>
+      <c r="C1276" t="s">
+        <v>3953</v>
+      </c>
+      <c r="D1276" t="s">
+        <v>4184</v>
+      </c>
+    </row>
+    <row r="1277" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1277" t="s">
+        <v>3954</v>
+      </c>
+      <c r="B1277" t="s">
+        <v>3129</v>
+      </c>
+      <c r="C1277" t="s">
+        <v>3955</v>
+      </c>
+      <c r="D1277" t="s">
+        <v>4185</v>
+      </c>
+    </row>
+    <row r="1278" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1278" t="s">
+        <v>3956</v>
+      </c>
+      <c r="B1278" t="s">
+        <v>3117</v>
+      </c>
+      <c r="C1278" t="s">
+        <v>3957</v>
+      </c>
+      <c r="D1278" t="s">
+        <v>4186</v>
+      </c>
+    </row>
+    <row r="1279" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1279" t="s">
+        <v>3958</v>
+      </c>
+      <c r="B1279" t="s">
+        <v>3157</v>
+      </c>
+      <c r="C1279" t="s">
+        <v>3959</v>
+      </c>
+      <c r="D1279" t="s">
+        <v>4187</v>
+      </c>
+    </row>
+    <row r="1280" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1280" t="s">
+        <v>3960</v>
+      </c>
+      <c r="B1280" t="s">
+        <v>3961</v>
+      </c>
+      <c r="C1280" t="s">
+        <v>3962</v>
+      </c>
+      <c r="D1280" t="s">
+        <v>4188</v>
+      </c>
+    </row>
+    <row r="1281" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1281" t="s">
+        <v>3963</v>
+      </c>
+      <c r="B1281" t="s">
+        <v>3017</v>
+      </c>
+      <c r="C1281" t="s">
+        <v>3964</v>
+      </c>
+      <c r="D1281" t="s">
+        <v>4189</v>
+      </c>
+    </row>
+    <row r="1282" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1282" t="s">
+        <v>3965</v>
+      </c>
+      <c r="B1282" t="s">
+        <v>3086</v>
+      </c>
+      <c r="C1282" t="s">
+        <v>3966</v>
+      </c>
+      <c r="D1282" t="s">
+        <v>4190</v>
+      </c>
+    </row>
+    <row r="1283" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1283" t="s">
+        <v>3967</v>
+      </c>
+      <c r="B1283" t="s">
+        <v>3968</v>
+      </c>
+      <c r="C1283" t="s">
+        <v>3969</v>
+      </c>
+      <c r="D1283" t="s">
+        <v>4191</v>
+      </c>
+    </row>
+    <row r="1284" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1284" t="s">
+        <v>3970</v>
+      </c>
+      <c r="B1284" t="s">
+        <v>3946</v>
+      </c>
+      <c r="C1284" t="s">
+        <v>3971</v>
+      </c>
+      <c r="D1284" t="s">
+        <v>4192</v>
+      </c>
+    </row>
+    <row r="1285" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1285" t="s">
+        <v>3972</v>
+      </c>
+      <c r="B1285" t="s">
+        <v>3124</v>
+      </c>
+      <c r="C1285" t="s">
+        <v>3973</v>
+      </c>
+      <c r="D1285" t="s">
+        <v>4193</v>
+      </c>
+    </row>
+    <row r="1286" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1286" t="s">
+        <v>3974</v>
+      </c>
+      <c r="B1286" t="s">
+        <v>3975</v>
+      </c>
+      <c r="C1286" t="s">
+        <v>3976</v>
+      </c>
+      <c r="D1286" t="s">
+        <v>4194</v>
+      </c>
+    </row>
+    <row r="1287" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1287" t="s">
+        <v>3977</v>
+      </c>
+      <c r="B1287" t="s">
+        <v>3978</v>
+      </c>
+      <c r="C1287" t="s">
+        <v>3979</v>
+      </c>
+      <c r="D1287" t="s">
+        <v>4195</v>
+      </c>
+    </row>
+    <row r="1288" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1288" t="s">
+        <v>3980</v>
+      </c>
+      <c r="B1288" t="s">
+        <v>3927</v>
+      </c>
+      <c r="C1288" t="s">
+        <v>3981</v>
+      </c>
+      <c r="D1288" t="s">
+        <v>4196</v>
+      </c>
+    </row>
+    <row r="1289" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1289" t="s">
+        <v>3982</v>
+      </c>
+      <c r="B1289" t="s">
+        <v>3014</v>
+      </c>
+      <c r="C1289" t="s">
+        <v>3983</v>
+      </c>
+      <c r="D1289" t="s">
+        <v>4197</v>
+      </c>
+    </row>
+    <row r="1290" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1290" t="s">
+        <v>3984</v>
+      </c>
+      <c r="B1290" t="s">
+        <v>3985</v>
+      </c>
+      <c r="C1290" t="s">
+        <v>3986</v>
+      </c>
+      <c r="D1290" t="s">
+        <v>4198</v>
+      </c>
+    </row>
+    <row r="1291" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1291" t="s">
+        <v>3987</v>
+      </c>
+      <c r="B1291" t="s">
+        <v>3172</v>
+      </c>
+      <c r="C1291" t="s">
+        <v>3988</v>
+      </c>
+      <c r="D1291" t="s">
+        <v>4199</v>
+      </c>
+    </row>
+    <row r="1292" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1292" t="s">
+        <v>3989</v>
+      </c>
+      <c r="B1292" t="s">
+        <v>3927</v>
+      </c>
+      <c r="C1292" t="s">
+        <v>3990</v>
+      </c>
+      <c r="D1292" t="s">
+        <v>4200</v>
+      </c>
+    </row>
+    <row r="1293" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1293" t="s">
+        <v>3991</v>
+      </c>
+      <c r="B1293" t="s">
+        <v>3992</v>
+      </c>
+      <c r="C1293" t="s">
+        <v>3993</v>
+      </c>
+      <c r="D1293" t="s">
+        <v>4201</v>
+      </c>
+    </row>
+    <row r="1294" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1294" t="s">
+        <v>3994</v>
+      </c>
+      <c r="B1294" t="s">
+        <v>3733</v>
+      </c>
+      <c r="C1294" t="s">
+        <v>3995</v>
+      </c>
+      <c r="D1294" t="s">
+        <v>4202</v>
+      </c>
+    </row>
+    <row r="1295" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1295" t="s">
+        <v>3996</v>
+      </c>
+      <c r="B1295" t="s">
+        <v>3997</v>
+      </c>
+      <c r="C1295" t="s">
+        <v>3998</v>
+      </c>
+      <c r="D1295" t="s">
+        <v>4203</v>
+      </c>
+    </row>
+    <row r="1296" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1296" t="s">
+        <v>3999</v>
+      </c>
+      <c r="B1296" t="s">
+        <v>4000</v>
+      </c>
+      <c r="C1296" t="s">
+        <v>4001</v>
+      </c>
+      <c r="D1296" t="s">
+        <v>4204</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1297" t="s">
+        <v>4002</v>
+      </c>
+      <c r="B1297" t="s">
+        <v>3169</v>
+      </c>
+      <c r="C1297" t="s">
+        <v>4003</v>
+      </c>
+      <c r="D1297" t="s">
+        <v>4205</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1298" t="s">
+        <v>4004</v>
+      </c>
+      <c r="B1298" t="s">
+        <v>3157</v>
+      </c>
+      <c r="C1298" t="s">
+        <v>4005</v>
+      </c>
+      <c r="D1298" t="s">
+        <v>4206</v>
+      </c>
+    </row>
+    <row r="1299" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1299" t="s">
+        <v>4006</v>
+      </c>
+      <c r="B1299" t="s">
+        <v>3175</v>
+      </c>
+      <c r="C1299" t="s">
+        <v>4007</v>
+      </c>
+      <c r="D1299" t="s">
+        <v>4207</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1300" t="s">
+        <v>4008</v>
+      </c>
+      <c r="B1300" t="s">
+        <v>4009</v>
+      </c>
+      <c r="C1300" t="s">
+        <v>4010</v>
+      </c>
+      <c r="D1300" t="s">
+        <v>4208</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1301" t="s">
+        <v>4011</v>
+      </c>
+      <c r="B1301" t="s">
+        <v>3172</v>
+      </c>
+      <c r="C1301" t="s">
+        <v>4012</v>
+      </c>
+      <c r="D1301" t="s">
+        <v>4209</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1302" t="s">
+        <v>4013</v>
+      </c>
+      <c r="B1302" t="s">
+        <v>4014</v>
+      </c>
+      <c r="C1302" t="s">
+        <v>4015</v>
+      </c>
+      <c r="D1302" t="s">
+        <v>4210</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1303" t="s">
+        <v>4016</v>
+      </c>
+      <c r="B1303" t="s">
+        <v>3717</v>
+      </c>
+      <c r="C1303" t="s">
+        <v>4017</v>
+      </c>
+      <c r="D1303" t="s">
+        <v>4211</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1304" t="s">
+        <v>4018</v>
+      </c>
+      <c r="B1304" t="s">
+        <v>4019</v>
+      </c>
+      <c r="C1304" t="s">
+        <v>4020</v>
+      </c>
+      <c r="D1304" t="s">
+        <v>4212</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1305" t="s">
+        <v>4021</v>
+      </c>
+      <c r="B1305" t="s">
+        <v>3774</v>
+      </c>
+      <c r="C1305" t="s">
+        <v>4022</v>
+      </c>
+      <c r="D1305" t="s">
+        <v>4213</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1306" t="s">
+        <v>4023</v>
+      </c>
+      <c r="B1306" t="s">
+        <v>4024</v>
+      </c>
+      <c r="C1306" t="s">
+        <v>4025</v>
+      </c>
+      <c r="D1306" t="s">
+        <v>4214</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1307" t="s">
+        <v>4026</v>
+      </c>
+      <c r="B1307" t="s">
+        <v>3749</v>
+      </c>
+      <c r="C1307" t="s">
+        <v>4027</v>
+      </c>
+      <c r="D1307" t="s">
+        <v>4215</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1308" t="s">
+        <v>4028</v>
+      </c>
+      <c r="B1308" t="s">
+        <v>3089</v>
+      </c>
+      <c r="C1308" t="s">
+        <v>4029</v>
+      </c>
+      <c r="D1308" t="s">
+        <v>4216</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1309" t="s">
+        <v>4030</v>
+      </c>
+      <c r="B1309" t="s">
+        <v>4031</v>
+      </c>
+      <c r="C1309" t="s">
+        <v>4032</v>
+      </c>
+      <c r="D1309" t="s">
+        <v>4217</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1310" t="s">
+        <v>4033</v>
+      </c>
+      <c r="B1310" t="s">
+        <v>4034</v>
+      </c>
+      <c r="C1310" t="s">
+        <v>4035</v>
+      </c>
+      <c r="D1310" t="s">
+        <v>4218</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1311" t="s">
+        <v>4036</v>
+      </c>
+      <c r="B1311" t="s">
+        <v>3749</v>
+      </c>
+      <c r="C1311" t="s">
+        <v>4037</v>
+      </c>
+      <c r="D1311" t="s">
+        <v>4219</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1312" t="s">
+        <v>4038</v>
+      </c>
+      <c r="B1312" t="s">
+        <v>3696</v>
+      </c>
+      <c r="C1312" t="s">
+        <v>4039</v>
+      </c>
+      <c r="D1312" t="s">
+        <v>4220</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1313" t="s">
+        <v>4040</v>
+      </c>
+      <c r="B1313" t="s">
+        <v>4041</v>
+      </c>
+      <c r="C1313" t="s">
+        <v>4042</v>
+      </c>
+      <c r="D1313" t="s">
+        <v>4221</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1314" t="s">
+        <v>4043</v>
+      </c>
+      <c r="B1314" t="s">
+        <v>3132</v>
+      </c>
+      <c r="C1314" t="s">
+        <v>4044</v>
+      </c>
+      <c r="D1314" t="s">
+        <v>4222</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1315" t="s">
+        <v>4045</v>
+      </c>
+      <c r="B1315" t="s">
+        <v>3922</v>
+      </c>
+      <c r="C1315" t="s">
+        <v>4046</v>
+      </c>
+      <c r="D1315" t="s">
+        <v>4223</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1316" t="s">
+        <v>4047</v>
+      </c>
+      <c r="B1316" t="s">
+        <v>3723</v>
+      </c>
+      <c r="C1316" t="s">
+        <v>4048</v>
+      </c>
+      <c r="D1316" t="s">
+        <v>4224</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1317" t="s">
+        <v>4049</v>
+      </c>
+      <c r="B1317" t="s">
+        <v>3756</v>
+      </c>
+      <c r="C1317" t="s">
+        <v>4050</v>
+      </c>
+      <c r="D1317" t="s">
+        <v>4225</v>
+      </c>
+    </row>
+    <row r="1318" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1318" t="s">
+        <v>4051</v>
+      </c>
+      <c r="B1318" t="s">
+        <v>3796</v>
+      </c>
+      <c r="C1318" t="s">
+        <v>4052</v>
+      </c>
+      <c r="D1318" t="s">
+        <v>4226</v>
+      </c>
+    </row>
+    <row r="1319" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1319" t="s">
+        <v>4053</v>
+      </c>
+      <c r="B1319" t="s">
+        <v>3035</v>
+      </c>
+      <c r="C1319" t="s">
+        <v>4054</v>
+      </c>
+      <c r="D1319" t="s">
+        <v>4227</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1320" t="s">
+        <v>4055</v>
+      </c>
+      <c r="B1320" t="s">
+        <v>3765</v>
+      </c>
+      <c r="C1320" t="s">
+        <v>4056</v>
+      </c>
+      <c r="D1320" t="s">
+        <v>4228</v>
+      </c>
+    </row>
+    <row r="1321" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1321" t="s">
+        <v>4057</v>
+      </c>
+      <c r="B1321" t="s">
+        <v>3047</v>
+      </c>
+      <c r="C1321" t="s">
+        <v>4058</v>
+      </c>
+      <c r="D1321" t="s">
+        <v>4229</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1322" t="s">
+        <v>4059</v>
+      </c>
+      <c r="B1322" t="s">
+        <v>3723</v>
+      </c>
+      <c r="C1322" t="s">
+        <v>4060</v>
+      </c>
+      <c r="D1322" t="s">
+        <v>4230</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1323" t="s">
+        <v>4061</v>
+      </c>
+      <c r="B1323" t="s">
+        <v>3839</v>
+      </c>
+      <c r="C1323" t="s">
+        <v>4062</v>
+      </c>
+      <c r="D1323" t="s">
+        <v>4231</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1324" t="s">
+        <v>4063</v>
+      </c>
+      <c r="B1324" t="s">
+        <v>3061</v>
+      </c>
+      <c r="C1324" t="s">
+        <v>4064</v>
+      </c>
+      <c r="D1324" t="s">
+        <v>4232</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1325" t="s">
+        <v>4065</v>
+      </c>
+      <c r="B1325" t="s">
+        <v>4066</v>
+      </c>
+      <c r="C1325" t="s">
+        <v>4067</v>
+      </c>
+      <c r="D1325" t="s">
+        <v>4233</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D956" xr:uid="{EE52D9B7-0D33-6C4B-ABD2-124A93043E14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>